<commit_message>
Excel: simplified summary block (day, current month, previous month, variation) with rolling month names
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UWVrfUbbvpriNVoC9v7Zjn
</commit_message>
<xml_diff>
--- a/volumes/suivi_cecafe.xlsx
+++ b/volumes/suivi_cecafe.xlsx
@@ -117,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,6 +140,15 @@
     <xf numFmtId="165" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -147,6 +156,22 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="001E8449"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="00C0392B"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -260,12 +285,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$9:$A$11</f>
+              <f>'Arabica'!$A$14:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$B$9:$B$11</f>
+              <f>'Arabica'!$B$14:$B$16</f>
             </numRef>
           </val>
         </ser>
@@ -288,12 +313,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$9:$A$11</f>
+              <f>'Arabica'!$A$14:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$D$9:$D$11</f>
+              <f>'Arabica'!$D$14:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -334,7 +359,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'Arabica'!$F$9:$F$11</f>
+              <f>'Arabica'!$F$14:$F$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -458,12 +483,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$35</f>
+              <f>'Robusta'!$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$B$35</f>
+              <f>'Robusta'!$B$40</f>
             </numRef>
           </val>
         </ser>
@@ -486,12 +511,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$35</f>
+              <f>'Robusta'!$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$C$35</f>
+              <f>'Robusta'!$C$40</f>
             </numRef>
           </val>
         </ser>
@@ -514,12 +539,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$35</f>
+              <f>'Robusta'!$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$D$35</f>
+              <f>'Robusta'!$D$40</f>
             </numRef>
           </val>
         </ser>
@@ -560,7 +585,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'Robusta'!$H$35</f>
+              <f>'Robusta'!$H$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -596,7 +621,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'Robusta'!$I$35</f>
+              <f>'Robusta'!$I$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -720,12 +745,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$15:$A$20</f>
+              <f>'Arabica'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$B$15:$B$20</f>
+              <f>'Arabica'!$B$20:$B$25</f>
             </numRef>
           </val>
         </ser>
@@ -748,12 +773,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$15:$A$20</f>
+              <f>'Arabica'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$C$15:$C$20</f>
+              <f>'Arabica'!$C$20:$C$25</f>
             </numRef>
           </val>
         </ser>
@@ -776,12 +801,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$15:$A$20</f>
+              <f>'Arabica'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$D$15:$D$20</f>
+              <f>'Arabica'!$D$20:$D$25</f>
             </numRef>
           </val>
         </ser>
@@ -878,12 +903,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$15:$A$20</f>
+              <f>'Arabica'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$E$15:$E$20</f>
+              <f>'Arabica'!$E$20:$E$25</f>
             </numRef>
           </val>
         </ser>
@@ -906,12 +931,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$15:$A$20</f>
+              <f>'Arabica'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$F$15:$F$20</f>
+              <f>'Arabica'!$F$20:$F$25</f>
             </numRef>
           </val>
         </ser>
@@ -934,12 +959,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$15:$A$20</f>
+              <f>'Arabica'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$G$15:$G$20</f>
+              <f>'Arabica'!$G$20:$G$25</f>
             </numRef>
           </val>
         </ser>
@@ -1036,12 +1061,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$25:$A$30</f>
+              <f>'Arabica'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$B$25:$B$30</f>
+              <f>'Arabica'!$B$30:$B$35</f>
             </numRef>
           </val>
         </ser>
@@ -1064,12 +1089,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$25:$A$30</f>
+              <f>'Arabica'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$C$25:$C$30</f>
+              <f>'Arabica'!$C$30:$C$35</f>
             </numRef>
           </val>
         </ser>
@@ -1092,12 +1117,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$25:$A$30</f>
+              <f>'Arabica'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$D$25:$D$30</f>
+              <f>'Arabica'!$D$30:$D$35</f>
             </numRef>
           </val>
         </ser>
@@ -1120,12 +1145,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$25:$A$30</f>
+              <f>'Arabica'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$E$25:$E$30</f>
+              <f>'Arabica'!$E$30:$E$35</f>
             </numRef>
           </val>
         </ser>
@@ -1148,12 +1173,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$25:$A$30</f>
+              <f>'Arabica'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$F$25:$F$30</f>
+              <f>'Arabica'!$F$30:$F$35</f>
             </numRef>
           </val>
         </ser>
@@ -1176,12 +1201,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$25:$A$30</f>
+              <f>'Arabica'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$G$25:$G$30</f>
+              <f>'Arabica'!$G$30:$G$35</f>
             </numRef>
           </val>
         </ser>
@@ -1278,12 +1303,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$35</f>
+              <f>'Arabica'!$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$B$35</f>
+              <f>'Arabica'!$B$40</f>
             </numRef>
           </val>
         </ser>
@@ -1306,12 +1331,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$35</f>
+              <f>'Arabica'!$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$C$35</f>
+              <f>'Arabica'!$C$40</f>
             </numRef>
           </val>
         </ser>
@@ -1334,12 +1359,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$35</f>
+              <f>'Arabica'!$A$40</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$D$35</f>
+              <f>'Arabica'!$D$40</f>
             </numRef>
           </val>
         </ser>
@@ -1380,7 +1405,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'Arabica'!$H$35</f>
+              <f>'Arabica'!$H$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1416,7 +1441,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'Arabica'!$I$35</f>
+              <f>'Arabica'!$I$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1540,12 +1565,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$9:$A$11</f>
+              <f>'Robusta'!$A$14:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$B$9:$B$11</f>
+              <f>'Robusta'!$B$14:$B$16</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1593,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$9:$A$11</f>
+              <f>'Robusta'!$A$14:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$D$9:$D$11</f>
+              <f>'Robusta'!$D$14:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -1614,7 +1639,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'Robusta'!$F$9:$F$11</f>
+              <f>'Robusta'!$F$14:$F$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1738,12 +1763,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$15:$A$20</f>
+              <f>'Robusta'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$B$15:$B$20</f>
+              <f>'Robusta'!$B$20:$B$25</f>
             </numRef>
           </val>
         </ser>
@@ -1766,12 +1791,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$15:$A$20</f>
+              <f>'Robusta'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$C$15:$C$20</f>
+              <f>'Robusta'!$C$20:$C$25</f>
             </numRef>
           </val>
         </ser>
@@ -1794,12 +1819,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$15:$A$20</f>
+              <f>'Robusta'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$D$15:$D$20</f>
+              <f>'Robusta'!$D$20:$D$25</f>
             </numRef>
           </val>
         </ser>
@@ -1896,12 +1921,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$15:$A$20</f>
+              <f>'Robusta'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$E$15:$E$20</f>
+              <f>'Robusta'!$E$20:$E$25</f>
             </numRef>
           </val>
         </ser>
@@ -1924,12 +1949,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$15:$A$20</f>
+              <f>'Robusta'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$F$15:$F$20</f>
+              <f>'Robusta'!$F$20:$F$25</f>
             </numRef>
           </val>
         </ser>
@@ -1952,12 +1977,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$15:$A$20</f>
+              <f>'Robusta'!$A$20:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$G$15:$G$20</f>
+              <f>'Robusta'!$G$20:$G$25</f>
             </numRef>
           </val>
         </ser>
@@ -2054,12 +2079,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$25:$A$30</f>
+              <f>'Robusta'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$B$25:$B$30</f>
+              <f>'Robusta'!$B$30:$B$35</f>
             </numRef>
           </val>
         </ser>
@@ -2082,12 +2107,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$25:$A$30</f>
+              <f>'Robusta'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$C$25:$C$30</f>
+              <f>'Robusta'!$C$30:$C$35</f>
             </numRef>
           </val>
         </ser>
@@ -2110,12 +2135,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$25:$A$30</f>
+              <f>'Robusta'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$D$25:$D$30</f>
+              <f>'Robusta'!$D$30:$D$35</f>
             </numRef>
           </val>
         </ser>
@@ -2138,12 +2163,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$25:$A$30</f>
+              <f>'Robusta'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$E$25:$E$30</f>
+              <f>'Robusta'!$E$30:$E$35</f>
             </numRef>
           </val>
         </ser>
@@ -2166,12 +2191,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$25:$A$30</f>
+              <f>'Robusta'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$F$25:$F$30</f>
+              <f>'Robusta'!$F$30:$F$35</f>
             </numRef>
           </val>
         </ser>
@@ -2194,12 +2219,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$25:$A$30</f>
+              <f>'Robusta'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$G$25:$G$30</f>
+              <f>'Robusta'!$G$30:$G$35</f>
             </numRef>
           </val>
         </ser>
@@ -2261,7 +2286,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -2283,7 +2308,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>31</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -2305,7 +2330,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>46</row>
+      <row>51</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -2327,7 +2352,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>66</row>
+      <row>71</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -2349,7 +2374,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>86</row>
+      <row>91</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -2376,7 +2401,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>6</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -2398,7 +2423,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>31</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -2420,7 +2445,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>46</row>
+      <row>51</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -2442,7 +2467,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>66</row>
+      <row>71</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -2464,7 +2489,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>86</row>
+      <row>91</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -4228,7 +4253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4297,704 +4322,795 @@
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>1. Par étape, toutes unités : jour J, veille, cumul du mois, variation % vs mois précédent</t>
+          <t>ARABICA — résumé (les noms de mois suivent la date affichée)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Mouvement du jour</t>
+        </is>
+      </c>
+      <c r="C8" s="3">
+        <f>CHOOSE(MONTH($B$4),"Janvier","Février","Mars","Avril","Mai","Juin","Juillet","Août","Septembre","Octobre","Novembre","Décembre")&amp;" "&amp;YEAR($B$4)</f>
+        <v/>
+      </c>
+      <c r="D8" s="3">
+        <f>CHOOSE(MONTH(DATE(YEAR($B$4),MONTH($B$4)+(-1),1)),"Janvier","Février","Mars","Avril","Mai","Juin","Juillet","Août","Septembre","Octobre","Novembre","Décembre")&amp;" "&amp;YEAR(DATE(YEAR($B$4),MONTH($B$4)+(-1),1))</f>
+        <v/>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Variation (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>ÉMISSION (certificats)</t>
+        </is>
+      </c>
+      <c r="B9" s="17">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="C9" s="17">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="D9" s="17">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="E9" s="18">
+        <f>IF(D9=0,NA(),C9/D9-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>EMBARQUE</t>
+        </is>
+      </c>
+      <c r="B10" s="17">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="C10" s="17">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="D10" s="17">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="E10" s="18">
+        <f>IF(D10=0,NA(),C10/D10-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Dédouanement = embarquement en total : même café vu par la douane. Colonne mois précédent = même période du mois précédent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>1. Par étape, toutes unités : jour J, veille, cumul du mois, variation % vs mois précédent</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t>Étape</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Jour J</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Veille</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Cumul mois</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Mois précédent (même période)</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="D13" s="3">
+        <f>"Cumul "&amp;CHOOSE(MONTH($B$4),"Janvier","Février","Mars","Avril","Mai","Juin","Juillet","Août","Septembre","Octobre","Novembre","Décembre")&amp;" "&amp;YEAR($B$4)</f>
+        <v/>
+      </c>
+      <c r="E13" s="3">
+        <f>CHOOSE(MONTH(DATE(YEAR($B$4),MONTH($B$4)+(-1),1)),"Janvier","Février","Mars","Avril","Mai","Juin","Juillet","Août","Septembre","Octobre","Novembre","Décembre")&amp;" "&amp;YEAR(DATE(YEAR($B$4),MONTH($B$4)+(-1),1))&amp;" (même période)"</f>
+        <v/>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Variation % vs mois précédent</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Certifiés − embarqués (cumul)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Certificats d'origine</t>
         </is>
       </c>
-      <c r="B9" s="16">
+      <c r="B14" s="19">
         <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
-      <c r="C9" s="16">
+      <c r="C14" s="19">
         <f>IF($B$5="",NA(),SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$5,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total"))</f>
         <v/>
       </c>
-      <c r="D9" s="16">
+      <c r="D14" s="19">
         <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
-      <c r="E9" s="16">
+      <c r="E14" s="19">
         <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
-      <c r="F9" s="17">
-        <f>IF(E9=0,NA(),D9/E9-1)</f>
-        <v/>
-      </c>
-      <c r="G9" s="16">
-        <f>D9-D11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Dédouanement</t>
-        </is>
-      </c>
-      <c r="B10" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="C10" s="16">
-        <f>IF($B$5="",NA(),SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$5,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total"))</f>
-        <v/>
-      </c>
-      <c r="D10" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="E10" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="F10" s="17">
-        <f>IF(E10=0,NA(),D10/E10-1)</f>
-        <v/>
-      </c>
-      <c r="G10" s="18" t="inlineStr">
-        <is>
-          <t>café vendu, pas encore parti</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Embarquement</t>
-        </is>
-      </c>
-      <c r="B11" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="C11" s="16">
-        <f>IF($B$5="",NA(),SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$5,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total"))</f>
-        <v/>
-      </c>
-      <c r="D11" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="E11" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="F11" s="17">
-        <f>IF(E11=0,NA(),D11/E11-1)</f>
-        <v/>
-      </c>
-      <c r="G11" s="7" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>2 et 3. Par port : mouvement du jour (graphique 2) et variation % du cumul vs mois précédent (graphique 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Port / unité</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Certificats J</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés J</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Embarqués J</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Var. % certificats</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Var. % dédouanés</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Var. % embarqués</t>
-        </is>
+      <c r="F14" s="20">
+        <f>IF(E14=0,NA(),D14/E14-1)</f>
+        <v/>
+      </c>
+      <c r="G14" s="19">
+        <f>D14-D16</f>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Santos</t>
-        </is>
-      </c>
-      <c r="B15" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="C15" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="D15" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="E15" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")-1)</f>
-        <v/>
-      </c>
-      <c r="F15" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")-1)</f>
-        <v/>
-      </c>
-      <c r="G15" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")-1)</f>
-        <v/>
+          <t>Dédouanement</t>
+        </is>
+      </c>
+      <c r="B15" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="C15" s="19">
+        <f>IF($B$5="",NA(),SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$5,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total"))</f>
+        <v/>
+      </c>
+      <c r="D15" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="E15" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="F15" s="20">
+        <f>IF(E15=0,NA(),D15/E15-1)</f>
+        <v/>
+      </c>
+      <c r="G15" s="21" t="inlineStr">
+        <is>
+          <t>café vendu, pas encore parti</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Vitória (ES)</t>
-        </is>
-      </c>
-      <c r="B16" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="C16" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="D16" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="E16" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
-        <v/>
-      </c>
-      <c r="F16" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
-        <v/>
-      </c>
-      <c r="G16" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Rio de Janeiro</t>
-        </is>
-      </c>
-      <c r="B17" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="C17" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="D17" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="E17" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")-1)</f>
-        <v/>
-      </c>
-      <c r="F17" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")-1)</f>
-        <v/>
-      </c>
-      <c r="G17" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")-1)</f>
-        <v/>
-      </c>
+          <t>Embarquement</t>
+        </is>
+      </c>
+      <c r="B16" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="C16" s="19">
+        <f>IF($B$5="",NA(),SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$5,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total"))</f>
+        <v/>
+      </c>
+      <c r="D16" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="E16" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="F16" s="20">
+        <f>IF(E16=0,NA(),D16/E16-1)</f>
+        <v/>
+      </c>
+      <c r="G16" s="7" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>REDEX / EADI Minas Gerais</t>
-        </is>
-      </c>
-      <c r="B18" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="C18" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="D18" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="E18" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")-1)</f>
-        <v/>
-      </c>
-      <c r="F18" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")-1)</f>
-        <v/>
-      </c>
-      <c r="G18" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")-1)</f>
-        <v/>
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>2 et 3. Par port : mouvement du jour (graphique 2) et variation % du cumul vs mois précédent (graphique 3)</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Salvador</t>
-        </is>
-      </c>
-      <c r="B19" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="C19" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="D19" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="E19" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")-1)</f>
-        <v/>
-      </c>
-      <c r="F19" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")-1)</f>
-        <v/>
-      </c>
-      <c r="G19" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")-1)</f>
-        <v/>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Port / unité</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Certificats J</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Dédouanés J</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Embarqués J</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Var. % certificats</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Var. % dédouanés</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Var. % embarqués</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Autres</t>
-        </is>
-      </c>
-      <c r="B20" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="C20" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="D20" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="E20" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")-1)</f>
-        <v/>
-      </c>
-      <c r="F20" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")-1)</f>
-        <v/>
-      </c>
-      <c r="G20" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")-1)</f>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B20" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="C20" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="D20" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="E20" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")-1)</f>
+        <v/>
+      </c>
+      <c r="F20" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")-1)</f>
+        <v/>
+      </c>
+      <c r="G20" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")-1)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Vitória et REDEX/EADI Minas n'ont pas de ligne « embarquement » sur la page : leur café part par Santos. #N/A = pas de valeur le mois précédent.</t>
-        </is>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Vitória (ES)</t>
+        </is>
+      </c>
+      <c r="B21" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="C21" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="E21" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
+        <v/>
+      </c>
+      <c r="F21" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
+        <v/>
+      </c>
+      <c r="G21" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="B22" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="C22" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="E22" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")-1)</f>
+        <v/>
+      </c>
+      <c r="F22" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")-1)</f>
+        <v/>
+      </c>
+      <c r="G22" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")-1)</f>
+        <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>4. Par port, cumul du mois (rouge) contre même période du mois précédent (bleu)</t>
-        </is>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>REDEX / EADI Minas Gerais</t>
+        </is>
+      </c>
+      <c r="B23" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="C23" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="D23" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="E23" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")-1)</f>
+        <v/>
+      </c>
+      <c r="F23" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")-1)</f>
+        <v/>
+      </c>
+      <c r="G23" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")-1)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Port / unité</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Certificats cumul</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Certificats mois préc.</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés cumul</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés mois préc.</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Embarqués cumul</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Embarqués mois préc.</t>
-        </is>
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="B24" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="C24" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="D24" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="E24" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")-1)</f>
+        <v/>
+      </c>
+      <c r="F24" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")-1)</f>
+        <v/>
+      </c>
+      <c r="G24" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")-1)</f>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Santos</t>
-        </is>
-      </c>
-      <c r="B25" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="C25" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="D25" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="E25" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="F25" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="G25" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+          <t>Autres</t>
+        </is>
+      </c>
+      <c r="B25" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
+        <v/>
+      </c>
+      <c r="C25" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
+        <v/>
+      </c>
+      <c r="D25" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
+        <v/>
+      </c>
+      <c r="E25" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")-1)</f>
+        <v/>
+      </c>
+      <c r="F25" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")-1)</f>
+        <v/>
+      </c>
+      <c r="G25" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")-1)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Vitória (ES)</t>
-        </is>
-      </c>
-      <c r="B26" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="C26" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="D26" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="E26" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="F26" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="G26" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Rio de Janeiro</t>
-        </is>
-      </c>
-      <c r="B27" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="C27" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="D27" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="E27" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="F27" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="G27" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Vitória et REDEX/EADI Minas n'ont pas de ligne « embarquement » sur la page : leur café part par Santos. #N/A = pas de valeur le mois précédent.</t>
+        </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>REDEX / EADI Minas Gerais</t>
-        </is>
-      </c>
-      <c r="B28" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="C28" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="D28" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="E28" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="F28" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="G28" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>4. Par port, cumul du mois (rouge) contre même période du mois précédent (bleu)</t>
+        </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>Salvador</t>
-        </is>
-      </c>
-      <c r="B29" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="C29" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="D29" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="E29" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="F29" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="G29" s="16">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Port / unité</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Certificats cumul</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Certificats mois préc.</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Dédouanés cumul</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Dédouanés mois préc.</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Embarqués cumul</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Embarqués mois préc.</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B30" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="C30" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="D30" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="E30" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="F30" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="G30" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Vitória (ES)</t>
+        </is>
+      </c>
+      <c r="B31" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="C31" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="D31" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="E31" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="F31" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="G31" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="B32" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="C32" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="D32" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="E32" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="F32" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="G32" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>REDEX / EADI Minas Gerais</t>
+        </is>
+      </c>
+      <c r="B33" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="C33" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="D33" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="E33" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="F33" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="G33" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="B34" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="C34" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="D34" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="E34" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="F34" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="G34" s="19">
+        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
           <t>Autres</t>
         </is>
       </c>
-      <c r="B30" s="16">
+      <c r="B35" s="19">
         <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
-      <c r="C30" s="16">
+      <c r="C35" s="19">
         <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
-      <c r="D30" s="16">
+      <c r="D35" s="19">
         <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
-      <c r="E30" s="16">
+      <c r="E35" s="19">
         <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
-      <c r="F30" s="16">
+      <c r="F35" s="19">
         <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
-      <c r="G30" s="16">
+      <c r="G35" s="19">
         <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>5. Historique jour par jour (toutes unités)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Certificats J</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>Dédouanés J</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>Embarqués J</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Certificats cumul</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Embarqués cumul</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Certifiés − embarqués</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>Var. % certificats vs mois préc.</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>Var. % embarqués vs mois préc.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="n">
+    <row r="40">
+      <c r="A40" s="6" t="n">
         <v>46269</v>
       </c>
-      <c r="B35" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="C35" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="D35" s="16">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="E35" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="F35" s="16">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="G35" s="16">
-        <f>E35-F35</f>
-        <v/>
-      </c>
-      <c r="H35" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")=0,NA(),E35/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")-1)</f>
-        <v/>
-      </c>
-      <c r="I35" s="17">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")=0,NA(),F35/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="B40" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="C40" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="D40" s="19">
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="E40" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="F40" s="19">
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="G40" s="19">
+        <f>E40-F40</f>
+        <v/>
+      </c>
+      <c r="H40" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")=0,NA(),E40/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")-1)</f>
+        <v/>
+      </c>
+      <c r="I40" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")=0,NA(),F40/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Le script build_xlsx.py ajoute une ligne par nouvelle journée. Si tu colles des jours à la main dans Donnees, ajoute aussi la date ici (colonne A), les formules de la ligne au-dessus se copient.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E9:E10">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -5006,7 +5122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5075,704 +5191,795 @@
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>1. Par étape, toutes unités : jour J, veille, cumul du mois, variation % vs mois précédent</t>
+          <t>ROBUSTA — résumé (les noms de mois suivent la date affichée)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Mouvement du jour</t>
+        </is>
+      </c>
+      <c r="C8" s="3">
+        <f>CHOOSE(MONTH($B$4),"Janvier","Février","Mars","Avril","Mai","Juin","Juillet","Août","Septembre","Octobre","Novembre","Décembre")&amp;" "&amp;YEAR($B$4)</f>
+        <v/>
+      </c>
+      <c r="D8" s="3">
+        <f>CHOOSE(MONTH(DATE(YEAR($B$4),MONTH($B$4)+(-1),1)),"Janvier","Février","Mars","Avril","Mai","Juin","Juillet","Août","Septembre","Octobre","Novembre","Décembre")&amp;" "&amp;YEAR(DATE(YEAR($B$4),MONTH($B$4)+(-1),1))</f>
+        <v/>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Variation (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>ÉMISSION (certificats)</t>
+        </is>
+      </c>
+      <c r="B9" s="17">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="C9" s="17">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="D9" s="17">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="E9" s="18">
+        <f>IF(D9=0,NA(),C9/D9-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>EMBARQUE</t>
+        </is>
+      </c>
+      <c r="B10" s="17">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="C10" s="17">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="D10" s="17">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="E10" s="18">
+        <f>IF(D10=0,NA(),C10/D10-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Dédouanement = embarquement en total : même café vu par la douane. Colonne mois précédent = même période du mois précédent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>1. Par étape, toutes unités : jour J, veille, cumul du mois, variation % vs mois précédent</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t>Étape</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Jour J</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Veille</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Cumul mois</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Mois précédent (même période)</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="D13" s="3">
+        <f>"Cumul "&amp;CHOOSE(MONTH($B$4),"Janvier","Février","Mars","Avril","Mai","Juin","Juillet","Août","Septembre","Octobre","Novembre","Décembre")&amp;" "&amp;YEAR($B$4)</f>
+        <v/>
+      </c>
+      <c r="E13" s="3">
+        <f>CHOOSE(MONTH(DATE(YEAR($B$4),MONTH($B$4)+(-1),1)),"Janvier","Février","Mars","Avril","Mai","Juin","Juillet","Août","Septembre","Octobre","Novembre","Décembre")&amp;" "&amp;YEAR(DATE(YEAR($B$4),MONTH($B$4)+(-1),1))&amp;" (même période)"</f>
+        <v/>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Variation % vs mois précédent</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Certifiés − embarqués (cumul)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Certificats d'origine</t>
         </is>
       </c>
-      <c r="B9" s="16">
+      <c r="B14" s="19">
         <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
-      <c r="C9" s="16">
+      <c r="C14" s="19">
         <f>IF($B$5="",NA(),SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$5,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total"))</f>
         <v/>
       </c>
-      <c r="D9" s="16">
+      <c r="D14" s="19">
         <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
-      <c r="E9" s="16">
+      <c r="E14" s="19">
         <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
-      <c r="F9" s="17">
-        <f>IF(E9=0,NA(),D9/E9-1)</f>
-        <v/>
-      </c>
-      <c r="G9" s="16">
-        <f>D9-D11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Dédouanement</t>
-        </is>
-      </c>
-      <c r="B10" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="C10" s="16">
-        <f>IF($B$5="",NA(),SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$5,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total"))</f>
-        <v/>
-      </c>
-      <c r="D10" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="E10" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="F10" s="17">
-        <f>IF(E10=0,NA(),D10/E10-1)</f>
-        <v/>
-      </c>
-      <c r="G10" s="18" t="inlineStr">
-        <is>
-          <t>café vendu, pas encore parti</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Embarquement</t>
-        </is>
-      </c>
-      <c r="B11" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="C11" s="16">
-        <f>IF($B$5="",NA(),SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$5,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total"))</f>
-        <v/>
-      </c>
-      <c r="D11" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="E11" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="F11" s="17">
-        <f>IF(E11=0,NA(),D11/E11-1)</f>
-        <v/>
-      </c>
-      <c r="G11" s="7" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>2 et 3. Par port : mouvement du jour (graphique 2) et variation % du cumul vs mois précédent (graphique 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Port / unité</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Certificats J</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés J</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Embarqués J</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Var. % certificats</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Var. % dédouanés</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Var. % embarqués</t>
-        </is>
+      <c r="F14" s="20">
+        <f>IF(E14=0,NA(),D14/E14-1)</f>
+        <v/>
+      </c>
+      <c r="G14" s="19">
+        <f>D14-D16</f>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Santos</t>
-        </is>
-      </c>
-      <c r="B15" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="C15" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="D15" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="E15" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")-1)</f>
-        <v/>
-      </c>
-      <c r="F15" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")-1)</f>
-        <v/>
-      </c>
-      <c r="G15" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")-1)</f>
-        <v/>
+          <t>Dédouanement</t>
+        </is>
+      </c>
+      <c r="B15" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="C15" s="19">
+        <f>IF($B$5="",NA(),SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$5,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total"))</f>
+        <v/>
+      </c>
+      <c r="D15" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="E15" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="F15" s="20">
+        <f>IF(E15=0,NA(),D15/E15-1)</f>
+        <v/>
+      </c>
+      <c r="G15" s="21" t="inlineStr">
+        <is>
+          <t>café vendu, pas encore parti</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Vitória (ES)</t>
-        </is>
-      </c>
-      <c r="B16" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="C16" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="D16" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="E16" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
-        <v/>
-      </c>
-      <c r="F16" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
-        <v/>
-      </c>
-      <c r="G16" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Rio de Janeiro</t>
-        </is>
-      </c>
-      <c r="B17" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="C17" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="D17" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="E17" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")-1)</f>
-        <v/>
-      </c>
-      <c r="F17" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")-1)</f>
-        <v/>
-      </c>
-      <c r="G17" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")-1)</f>
-        <v/>
-      </c>
+          <t>Embarquement</t>
+        </is>
+      </c>
+      <c r="B16" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="C16" s="19">
+        <f>IF($B$5="",NA(),SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$5,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total"))</f>
+        <v/>
+      </c>
+      <c r="D16" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="E16" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="F16" s="20">
+        <f>IF(E16=0,NA(),D16/E16-1)</f>
+        <v/>
+      </c>
+      <c r="G16" s="7" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>REDEX / EADI Minas Gerais</t>
-        </is>
-      </c>
-      <c r="B18" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="C18" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="D18" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="E18" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")-1)</f>
-        <v/>
-      </c>
-      <c r="F18" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")-1)</f>
-        <v/>
-      </c>
-      <c r="G18" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")-1)</f>
-        <v/>
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>2 et 3. Par port : mouvement du jour (graphique 2) et variation % du cumul vs mois précédent (graphique 3)</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Salvador</t>
-        </is>
-      </c>
-      <c r="B19" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="C19" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="D19" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="E19" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")-1)</f>
-        <v/>
-      </c>
-      <c r="F19" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")-1)</f>
-        <v/>
-      </c>
-      <c r="G19" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")-1)</f>
-        <v/>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Port / unité</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Certificats J</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Dédouanés J</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Embarqués J</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Var. % certificats</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Var. % dédouanés</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Var. % embarqués</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Autres</t>
-        </is>
-      </c>
-      <c r="B20" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="C20" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="D20" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="E20" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")-1)</f>
-        <v/>
-      </c>
-      <c r="F20" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")-1)</f>
-        <v/>
-      </c>
-      <c r="G20" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")-1)</f>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B20" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="C20" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="D20" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="E20" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")-1)</f>
+        <v/>
+      </c>
+      <c r="F20" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")-1)</f>
+        <v/>
+      </c>
+      <c r="G20" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")-1)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Vitória et REDEX/EADI Minas n'ont pas de ligne « embarquement » sur la page : leur café part par Santos. #N/A = pas de valeur le mois précédent.</t>
-        </is>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Vitória (ES)</t>
+        </is>
+      </c>
+      <c r="B21" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="C21" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="E21" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
+        <v/>
+      </c>
+      <c r="F21" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
+        <v/>
+      </c>
+      <c r="G21" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="B22" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="C22" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="E22" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")-1)</f>
+        <v/>
+      </c>
+      <c r="F22" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")-1)</f>
+        <v/>
+      </c>
+      <c r="G22" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")-1)</f>
+        <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>4. Par port, cumul du mois (rouge) contre même période du mois précédent (bleu)</t>
-        </is>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>REDEX / EADI Minas Gerais</t>
+        </is>
+      </c>
+      <c r="B23" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="C23" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="D23" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="E23" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")-1)</f>
+        <v/>
+      </c>
+      <c r="F23" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")-1)</f>
+        <v/>
+      </c>
+      <c r="G23" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")-1)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Port / unité</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Certificats cumul</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Certificats mois préc.</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés cumul</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés mois préc.</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Embarqués cumul</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Embarqués mois préc.</t>
-        </is>
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="B24" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="C24" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="D24" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="E24" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")-1)</f>
+        <v/>
+      </c>
+      <c r="F24" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")-1)</f>
+        <v/>
+      </c>
+      <c r="G24" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")-1)</f>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Santos</t>
-        </is>
-      </c>
-      <c r="B25" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="C25" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="D25" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="E25" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="F25" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
-        <v/>
-      </c>
-      <c r="G25" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+          <t>Autres</t>
+        </is>
+      </c>
+      <c r="B25" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
+        <v/>
+      </c>
+      <c r="C25" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
+        <v/>
+      </c>
+      <c r="D25" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
+        <v/>
+      </c>
+      <c r="E25" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")-1)</f>
+        <v/>
+      </c>
+      <c r="F25" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")-1)</f>
+        <v/>
+      </c>
+      <c r="G25" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")=0,NA(),SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")-1)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Vitória (ES)</t>
-        </is>
-      </c>
-      <c r="B26" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="C26" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="D26" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="E26" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="F26" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="G26" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Rio de Janeiro</t>
-        </is>
-      </c>
-      <c r="B27" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="C27" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="D27" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="E27" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="F27" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="G27" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Vitória et REDEX/EADI Minas n'ont pas de ligne « embarquement » sur la page : leur café part par Santos. #N/A = pas de valeur le mois précédent.</t>
+        </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>REDEX / EADI Minas Gerais</t>
-        </is>
-      </c>
-      <c r="B28" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="C28" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="D28" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="E28" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="F28" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="G28" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>4. Par port, cumul du mois (rouge) contre même période du mois précédent (bleu)</t>
+        </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>Salvador</t>
-        </is>
-      </c>
-      <c r="B29" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="C29" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="D29" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="E29" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="F29" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="G29" s="16">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Port / unité</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Certificats cumul</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Certificats mois préc.</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Dédouanés cumul</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Dédouanés mois préc.</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Embarqués cumul</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Embarqués mois préc.</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B30" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="C30" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="D30" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="E30" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="F30" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+      <c r="G30" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Vitória (ES)</t>
+        </is>
+      </c>
+      <c r="B31" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="C31" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="D31" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="E31" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="F31" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+      <c r="G31" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="B32" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="C32" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="D32" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="E32" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="F32" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+      <c r="G32" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>REDEX / EADI Minas Gerais</t>
+        </is>
+      </c>
+      <c r="B33" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="C33" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="D33" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="E33" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="F33" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+      <c r="G33" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="B34" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="C34" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="D34" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="E34" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="F34" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+      <c r="G34" s="19">
+        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
           <t>Autres</t>
         </is>
       </c>
-      <c r="B30" s="16">
+      <c r="B35" s="19">
         <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
-      <c r="C30" s="16">
+      <c r="C35" s="19">
         <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
-      <c r="D30" s="16">
+      <c r="D35" s="19">
         <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
-      <c r="E30" s="16">
+      <c r="E35" s="19">
         <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
-      <c r="F30" s="16">
+      <c r="F35" s="19">
         <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
-      <c r="G30" s="16">
+      <c r="G35" s="19">
         <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>5. Historique jour par jour (toutes unités)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Certificats J</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>Dédouanés J</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>Embarqués J</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Certificats cumul</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Embarqués cumul</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Certifiés − embarqués</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>Var. % certificats vs mois préc.</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>Var. % embarqués vs mois préc.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="n">
+    <row r="40">
+      <c r="A40" s="6" t="n">
         <v>46269</v>
       </c>
-      <c r="B35" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="C35" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="D35" s="16">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="E35" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="F35" s="16">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="G35" s="16">
-        <f>E35-F35</f>
-        <v/>
-      </c>
-      <c r="H35" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")=0,NA(),E35/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")-1)</f>
-        <v/>
-      </c>
-      <c r="I35" s="17">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")=0,NA(),F35/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A35,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="B40" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="C40" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="D40" s="19">
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="E40" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="F40" s="19">
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
+        <v/>
+      </c>
+      <c r="G40" s="19">
+        <f>E40-F40</f>
+        <v/>
+      </c>
+      <c r="H40" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")=0,NA(),E40/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")-1)</f>
+        <v/>
+      </c>
+      <c r="I40" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")=0,NA(),F40/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Le script build_xlsx.py ajoute une ligne par nouvelle journée. Si tu colles des jours à la main dans Donnees, ajoute aussi la date ici (colonne A), les formules de la ligne au-dessus se copient.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E9:E10">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel: chart 1 without cumulative, drop per-port cumulative block
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UWVrfUbbvpriNVoC9v7Zjn
</commit_message>
<xml_diff>
--- a/volumes/suivi_cecafe.xlsx
+++ b/volumes/suivi_cecafe.xlsx
@@ -256,7 +256,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Arabica — mouvement du jour (rouge), cumul du mois (vert), variation % vs mois précédent (bleu, axe droit)</a:t>
+              <a:t>Arabica — mouvement du jour (rouge) et variation % du cumul vs mois précédent (bleu, axe droit)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -294,34 +294,6 @@
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <v>Cumul du mois</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="2E8B57"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="2E8B57"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Arabica'!$A$14:$A$16</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Arabica'!$D$14:$D$16</f>
-            </numRef>
-          </val>
-        </ser>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -329,8 +301,8 @@
       <lineChart>
         <grouping val="standard"/>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="1"/>
+          <order val="1"/>
           <tx>
             <v>Variation % vs mois précédent</v>
           </tx>
@@ -360,268 +332,6 @@
           <val>
             <numRef>
               <f>'Arabica'!$F$14:$F$16</f>
-            </numRef>
-          </val>
-          <smooth val="0"/>
-        </ser>
-        <axId val="10"/>
-        <axId val="200"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>sacs 60 kg</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-      <valAx>
-        <axId val="200"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>variation vs mois précédent</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-        <crosses val="max"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="b"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Robusta — historique quotidien (rouges) et variation % vs mois précédent (bleus, axe droit)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <v>Certificats J</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="C0392B"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="C0392B"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Robusta'!$A$40</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Robusta'!$B$40</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <v>Dédouanés J</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="E07B6B"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="E07B6B"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Robusta'!$A$40</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Robusta'!$C$40</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <v>Embarqués J</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="F2B8B0"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="F2B8B0"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Robusta'!$A$40</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Robusta'!$D$40</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <v>Var. % certificats</v>
-          </tx>
-          <spPr>
-            <a:ln w="22000">
-              <a:solidFill>
-                <a:srgbClr val="1F4E9C"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="circle"/>
-            <size val="6"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="1F4E9C"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="1F4E9C"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <val>
-            <numRef>
-              <f>'Robusta'!$H$40</f>
-            </numRef>
-          </val>
-          <smooth val="0"/>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <tx>
-            <v>Var. % embarqués</v>
-          </tx>
-          <spPr>
-            <a:ln w="22000">
-              <a:solidFill>
-                <a:srgbClr val="9DC3F0"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="circle"/>
-            <size val="6"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="9DC3F0"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="9DC3F0"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <val>
-            <numRef>
-              <f>'Robusta'!$I$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1032,248 +742,6 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Arabica — cumul du mois (rouges) vs même période du mois précédent (bleus)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <v>Certificats cumul</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="C0392B"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="C0392B"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Arabica'!$A$30:$A$35</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Arabica'!$B$30:$B$35</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <v>Certificats mois préc.</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="1F4E9C"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="1F4E9C"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Arabica'!$A$30:$A$35</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Arabica'!$C$30:$C$35</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <v>Dédouanés cumul</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="E07B6B"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="E07B6B"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Arabica'!$A$30:$A$35</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Arabica'!$D$30:$D$35</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <v>Dédouanés mois préc.</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="2F6FBF"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="2F6FBF"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Arabica'!$A$30:$A$35</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Arabica'!$E$30:$E$35</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <tx>
-            <v>Embarqués cumul</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="F2B8B0"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="F2B8B0"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Arabica'!$A$30:$A$35</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Arabica'!$F$30:$F$35</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="5"/>
-          <order val="5"/>
-          <tx>
-            <v>Embarqués mois préc.</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="9DC3F0"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="9DC3F0"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Arabica'!$A$30:$A$35</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Arabica'!$G$30:$G$35</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>sacs 60 kg</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="b"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
               <a:t>Arabica — historique quotidien (rouges) et variation % vs mois précédent (bleus, axe droit)</a:t>
             </a:r>
           </a:p>
@@ -1303,12 +771,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$40</f>
+              <f>'Arabica'!$A$30</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$B$40</f>
+              <f>'Arabica'!$B$30</f>
             </numRef>
           </val>
         </ser>
@@ -1331,12 +799,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$40</f>
+              <f>'Arabica'!$A$30</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$C$40</f>
+              <f>'Arabica'!$C$30</f>
             </numRef>
           </val>
         </ser>
@@ -1359,12 +827,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Arabica'!$A$40</f>
+              <f>'Arabica'!$A$30</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Arabica'!$D$40</f>
+              <f>'Arabica'!$D$30</f>
             </numRef>
           </val>
         </ser>
@@ -1405,7 +873,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'Arabica'!$H$40</f>
+              <f>'Arabica'!$H$30</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1441,7 +909,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'Arabica'!$I$40</f>
+              <f>'Arabica'!$I$30</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1524,7 +992,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1536,7 +1004,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Robusta — mouvement du jour (rouge), cumul du mois (vert), variation % vs mois précédent (bleu, axe droit)</a:t>
+              <a:t>Robusta — mouvement du jour (rouge) et variation % du cumul vs mois précédent (bleu, axe droit)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -1574,34 +1042,6 @@
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <v>Cumul du mois</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="2E8B57"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="2E8B57"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Robusta'!$A$14:$A$16</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Robusta'!$D$14:$D$16</f>
-            </numRef>
-          </val>
-        </ser>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -1609,8 +1049,8 @@
       <lineChart>
         <grouping val="standard"/>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="1"/>
+          <order val="1"/>
           <tx>
             <v>Variation % vs mois précédent</v>
           </tx>
@@ -1722,7 +1162,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1880,7 +1320,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -2038,7 +1478,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -2050,7 +1490,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Robusta — cumul du mois (rouges) vs même période du mois précédent (bleus)</a:t>
+              <a:t>Robusta — historique quotidien (rouges) et variation % vs mois précédent (bleus, axe droit)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -2064,7 +1504,7 @@
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <v>Certificats cumul</v>
+            <v>Certificats J</v>
           </tx>
           <spPr>
             <a:solidFill>
@@ -2079,12 +1519,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$30:$A$35</f>
+              <f>'Robusta'!$A$30</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$B$30:$B$35</f>
+              <f>'Robusta'!$B$30</f>
             </numRef>
           </val>
         </ser>
@@ -2092,35 +1532,7 @@
           <idx val="1"/>
           <order val="1"/>
           <tx>
-            <v>Certificats mois préc.</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="1F4E9C"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="1F4E9C"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Robusta'!$A$30:$A$35</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Robusta'!$C$30:$C$35</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <v>Dédouanés cumul</v>
+            <v>Dédouanés J</v>
           </tx>
           <spPr>
             <a:solidFill>
@@ -2135,48 +1547,20 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$30:$A$35</f>
+              <f>'Robusta'!$A$30</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$D$30:$D$35</f>
+              <f>'Robusta'!$C$30</f>
             </numRef>
           </val>
         </ser>
         <ser>
-          <idx val="3"/>
-          <order val="3"/>
+          <idx val="2"/>
+          <order val="2"/>
           <tx>
-            <v>Dédouanés mois préc.</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="2F6FBF"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="2F6FBF"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Robusta'!$A$30:$A$35</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Robusta'!$E$30:$E$35</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <tx>
-            <v>Embarqués cumul</v>
+            <v>Embarqués J</v>
           </tx>
           <spPr>
             <a:solidFill>
@@ -2191,40 +1575,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Robusta'!$A$30:$A$35</f>
+              <f>'Robusta'!$A$30</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Robusta'!$F$30:$F$35</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="5"/>
-          <order val="5"/>
-          <tx>
-            <v>Embarqués mois préc.</v>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="9DC3F0"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="9DC3F0"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Robusta'!$A$30:$A$35</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Robusta'!$G$30:$G$35</f>
+              <f>'Robusta'!$D$30</f>
             </numRef>
           </val>
         </ser>
@@ -2232,6 +1588,83 @@
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <v>Var. % certificats</v>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="1F4E9C"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F4E9C"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1F4E9C"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Robusta'!$H$30</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <v>Var. % embarqués</v>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="9DC3F0"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="9DC3F0"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="9DC3F0"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Robusta'!$I$30</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="200"/>
+      </lineChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -2269,6 +1702,33 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="200"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>variation vs mois précédent</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <legend>
@@ -2352,7 +1812,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>71</row>
+      <row>51</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -2365,28 +1825,6 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId4"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>8</col>
-      <colOff>0</colOff>
-      <row>91</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7200000" cy="3420000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="5" name="Chart 5"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2467,7 +1905,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>71</row>
+      <row>51</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="3420000"/>
@@ -2480,28 +1918,6 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId4"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>8</col>
-      <colOff>0</colOff>
-      <row>91</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7200000" cy="3420000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="5" name="Chart 5"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4253,7 +3669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4777,36 +4193,36 @@
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>4. Par port, cumul du mois (rouge) contre même période du mois précédent (bleu)</t>
+          <t>4. Historique jour par jour (toutes unités)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Port / unité</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
+          <t>Certificats J</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Dédouanés J</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Embarqués J</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
           <t>Certificats cumul</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Certificats mois préc.</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés cumul</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés mois préc.</t>
-        </is>
-      </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Embarqués cumul</t>
@@ -4814,289 +4230,59 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Embarqués mois préc.</t>
+          <t>Certifiés − embarqués</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Var. % certificats vs mois préc.</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Var. % embarqués vs mois préc.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Santos</t>
-        </is>
+      <c r="A30" s="6" t="n">
+        <v>46269</v>
       </c>
       <c r="B30" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
       <c r="C30" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
       <c r="D30" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
       <c r="E30" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
       <c r="F30" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
       <c r="G30" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>E30-F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")=0,NA(),E30/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")-1)</f>
+        <v/>
+      </c>
+      <c r="I30" s="20">
+        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")=0,NA(),F30/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")-1)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>Vitória (ES)</t>
-        </is>
-      </c>
-      <c r="B31" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="C31" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="D31" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="E31" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="F31" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="G31" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Rio de Janeiro</t>
-        </is>
-      </c>
-      <c r="B32" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="C32" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="D32" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="E32" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="F32" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="G32" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>REDEX / EADI Minas Gerais</t>
-        </is>
-      </c>
-      <c r="B33" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="C33" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="D33" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="E33" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="F33" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="G33" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>Salvador</t>
-        </is>
-      </c>
-      <c r="B34" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="C34" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="D34" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="E34" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="F34" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="G34" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>Autres</t>
-        </is>
-      </c>
-      <c r="B35" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="C35" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="D35" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="E35" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="F35" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="G35" s="19">
-        <f>SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="15" t="inlineStr">
-        <is>
-          <t>5. Historique jour par jour (toutes unités)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Certificats J</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés J</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>Embarqués J</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Certificats cumul</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>Embarqués cumul</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Certifiés − embarqués</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>Var. % certificats vs mois préc.</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>Var. % embarqués vs mois préc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="n">
-        <v>46269</v>
-      </c>
-      <c r="B40" s="19">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="C40" s="19">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="D40" s="19">
-        <f>SUMIFS(Donnees!$E$2:$E$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="E40" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="F40" s="19">
-        <f>SUMIFS(Donnees!$I$2:$I$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="G40" s="19">
-        <f>E40-F40</f>
-        <v/>
-      </c>
-      <c r="H40" s="20">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")=0,NA(),E40/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")-1)</f>
-        <v/>
-      </c>
-      <c r="I40" s="20">
-        <f>IF(SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")=0,NA(),F40/SUMIFS(Donnees!$M$2:$M$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Le script build_xlsx.py ajoute une ligne par nouvelle journée. Si tu colles des jours à la main dans Donnees, ajoute aussi la date ici (colonne A), les formules de la ligne au-dessus se copient.</t>
         </is>
@@ -5122,7 +4308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5646,36 +4832,36 @@
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>4. Par port, cumul du mois (rouge) contre même période du mois précédent (bleu)</t>
+          <t>4. Historique jour par jour (toutes unités)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Port / unité</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
+          <t>Certificats J</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Dédouanés J</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Embarqués J</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
           <t>Certificats cumul</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Certificats mois préc.</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés cumul</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés mois préc.</t>
-        </is>
-      </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Embarqués cumul</t>
@@ -5683,289 +4869,59 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Embarqués mois préc.</t>
+          <t>Certifiés − embarqués</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Var. % certificats vs mois préc.</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Var. % embarqués vs mois préc.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Santos</t>
-        </is>
+      <c r="A30" s="6" t="n">
+        <v>46269</v>
       </c>
       <c r="B30" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
       <c r="C30" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
       <c r="D30" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
       <c r="E30" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
       <c r="F30" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
         <v/>
       </c>
       <c r="G30" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"santos")</f>
+        <f>E30-F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")=0,NA(),E30/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")-1)</f>
+        <v/>
+      </c>
+      <c r="I30" s="20">
+        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")=0,NA(),F30/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A30,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")-1)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>Vitória (ES)</t>
-        </is>
-      </c>
-      <c r="B31" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="C31" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="D31" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="E31" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="F31" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-      <c r="G31" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"vitoria")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>Rio de Janeiro</t>
-        </is>
-      </c>
-      <c r="B32" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="C32" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="D32" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="E32" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="F32" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-      <c r="G32" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"rio")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>REDEX / EADI Minas Gerais</t>
-        </is>
-      </c>
-      <c r="B33" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="C33" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="D33" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="E33" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="F33" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-      <c r="G33" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"minas")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>Salvador</t>
-        </is>
-      </c>
-      <c r="B34" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="C34" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="D34" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="E34" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="F34" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-      <c r="G34" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"salvador")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>Autres</t>
-        </is>
-      </c>
-      <c r="B35" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="C35" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="D35" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="E35" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="F35" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-      <c r="G35" s="19">
-        <f>SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$B$4,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"others")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="15" t="inlineStr">
-        <is>
-          <t>5. Historique jour par jour (toutes unités)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Certificats J</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Dédouanés J</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>Embarqués J</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Certificats cumul</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>Embarqués cumul</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Certifiés − embarqués</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>Var. % certificats vs mois préc.</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>Var. % embarqués vs mois préc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="n">
-        <v>46269</v>
-      </c>
-      <c r="B40" s="19">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="C40" s="19">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"customs",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="D40" s="19">
-        <f>SUMIFS(Donnees!$F$2:$F$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="E40" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="F40" s="19">
-        <f>SUMIFS(Donnees!$J$2:$J$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")</f>
-        <v/>
-      </c>
-      <c r="G40" s="19">
-        <f>E40-F40</f>
-        <v/>
-      </c>
-      <c r="H40" s="20">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")=0,NA(),E40/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"certificates",Donnees!$C$2:$C$5000,"total")-1)</f>
-        <v/>
-      </c>
-      <c r="I40" s="20">
-        <f>IF(SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")=0,NA(),F40/SUMIFS(Donnees!$N$2:$N$5000,Donnees!$A$2:$A$5000,$A40,Donnees!$B$2:$B$5000,"shipment",Donnees!$C$2:$C$5000,"total")-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Le script build_xlsx.py ajoute une ligne par nouvelle journée. Si tu colles des jours à la main dans Donnees, ajoute aussi la date ici (colonne A), les formules de la ligne au-dessus se copient.</t>
         </is>

</xml_diff>